<commit_message>
Mit I2C Koppler neu
</commit_message>
<xml_diff>
--- a/Bauteillisten/Bauteile.xlsx
+++ b/Bauteillisten/Bauteile.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maria\Documents\Uni\Semester 6\Projektarbeit\Bauteillisten\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maria\Documents\Uni\Semester 6\Projektarbeit\active-balancing\Bauteillisten\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{931B9965-787F-4E57-855C-5AE586770B1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D89B061D-C9A0-4482-BDA5-EAE57A1C4FBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{F1FF9425-874B-4F4E-A494-92F342246896}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{F1FF9425-874B-4F4E-A494-92F342246896}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="84">
   <si>
     <t>Bezeichnung</t>
   </si>
@@ -276,6 +276,21 @@
   </si>
   <si>
     <t>2x benötigt</t>
+  </si>
+  <si>
+    <t>ADuM1250</t>
+  </si>
+  <si>
+    <t>ADUM1250ARZ-RL7</t>
+  </si>
+  <si>
+    <t>4x -&gt; auf jeder Seite 2</t>
+  </si>
+  <si>
+    <t>2x jeweils auf jeder seite 1</t>
+  </si>
+  <si>
+    <t>Isolated I2C Digital analog wandler  DAC</t>
   </si>
 </sst>
 </file>
@@ -295,12 +310,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -315,10 +336,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="8" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -653,7 +676,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9F06275-B373-4E0F-A893-36D48C0A1B98}">
-  <dimension ref="A1:R35"/>
+  <dimension ref="A1:R42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.35">
@@ -1014,47 +1037,129 @@
         <v>1.39</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A33" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="F33" s="3"/>
+      <c r="G33" s="4">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="H33" s="3"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A34" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B34" s="3"/>
+      <c r="C34" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D34" s="3"/>
+      <c r="E34" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="F34" s="3"/>
+      <c r="G34" s="4">
+        <v>0.09</v>
+      </c>
+      <c r="H34" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A35" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B35" s="3"/>
+      <c r="C35" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D35" s="3"/>
+      <c r="E35" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F35" s="3"/>
+      <c r="G35" s="4">
+        <v>0.09</v>
+      </c>
+      <c r="H35" s="3"/>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A39" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="E33" t="s">
-        <v>70</v>
-      </c>
-      <c r="G33" s="1">
-        <v>1.0900000000000001</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
+      <c r="B39" s="3"/>
+      <c r="C39" s="3"/>
+      <c r="D39" s="3"/>
+      <c r="E39" s="3"/>
+      <c r="F39" s="3"/>
+      <c r="G39" s="3"/>
+      <c r="H39" s="3"/>
+      <c r="I39" s="3"/>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A40" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B40" s="3"/>
+      <c r="C40" s="3"/>
+      <c r="D40" s="3"/>
+      <c r="E40" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+      <c r="H40" s="3"/>
+      <c r="I40" s="3"/>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A41" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C34" t="s">
+      <c r="B41" s="3"/>
+      <c r="C41" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="E34" t="s">
+      <c r="D41" s="3"/>
+      <c r="E41" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="G34" s="1">
+      <c r="F41" s="3"/>
+      <c r="G41" s="4">
         <v>0.09</v>
       </c>
-      <c r="H34" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
+      <c r="H41" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="I41" s="3"/>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A42" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="C35" t="s">
+      <c r="B42" s="3"/>
+      <c r="C42" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="E35" t="s">
+      <c r="D42" s="3"/>
+      <c r="E42" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="G35" s="1">
+      <c r="F42" s="3"/>
+      <c r="G42" s="4">
         <v>0.09</v>
       </c>
+      <c r="H42" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="I42" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>